<commit_message>
Reworked ESP_IMU_Board to fix the regulator issue, some layout inconsistancies, and footprint mismatches.
</commit_message>
<xml_diff>
--- a/Hardware/Documentation/ESP_IMU_Board_BOM.xlsx
+++ b/Hardware/Documentation/ESP_IMU_Board_BOM.xlsx
@@ -1,26 +1,73 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/georgetrupiano/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\George\Documents\GitHub\ORA\Hardware\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{3F386D18-7BF4-5D40-83A4-0155AA6E5A0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{278926C0-621C-4F9F-BC92-7B3CB319E766}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="17280" windowHeight="20040" xr2:uid="{816A1135-95D1-CA46-8F76-FE45BE9CB508}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{816A1135-95D1-CA46-8F76-FE45BE9CB508}"/>
   </bookViews>
   <sheets>
-    <sheet name="ESP_IMU_Board1" sheetId="1" r:id="rId1"/>
+    <sheet name="ESP_IMU_Board" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>George</author>
+  </authors>
+  <commentList>
+    <comment ref="G10" authorId="0" shapeId="0" xr:uid="{AF85A7AA-7D37-4499-AA52-B52E8AC4D249}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>George:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+I'm doing the highest cost per unit so it may be lower if it is decided to buy in bulk.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="82">
   <si>
     <t>Reference</t>
   </si>
@@ -34,12 +81,6 @@
     <t>10uF</t>
   </si>
   <si>
-    <t>C2</t>
-  </si>
-  <si>
-    <t>22uF</t>
-  </si>
-  <si>
     <t>C5,C7,C11,C12,C13,C14</t>
   </si>
   <si>
@@ -55,12 +96,6 @@
     <t>LED</t>
   </si>
   <si>
-    <t>J1</t>
-  </si>
-  <si>
-    <t>USB_C_Receptacle_USB2.0_14P</t>
-  </si>
-  <si>
     <t>J2</t>
   </si>
   <si>
@@ -112,18 +147,6 @@
     <t>R11</t>
   </si>
   <si>
-    <t>SW1</t>
-  </si>
-  <si>
-    <t>Enable</t>
-  </si>
-  <si>
-    <t>SW2</t>
-  </si>
-  <si>
-    <t>Boot</t>
-  </si>
-  <si>
     <t>U1</t>
   </si>
   <si>
@@ -133,9 +156,6 @@
     <t>U2</t>
   </si>
   <si>
-    <t>AMS1117-3.3</t>
-  </si>
-  <si>
     <t>U3</t>
   </si>
   <si>
@@ -148,51 +168,12 @@
     <t>Link</t>
   </si>
   <si>
-    <t>C1</t>
-  </si>
-  <si>
     <t>C6,C8</t>
   </si>
   <si>
     <t>Notes</t>
   </si>
   <si>
-    <t>Polarized capactor</t>
-  </si>
-  <si>
-    <t>0805W106K250CC</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/products/detail/nextgen-components/0805W106K250CC/18676983</t>
-  </si>
-  <si>
-    <t>0805B104K500BD</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/products/detail/nextgen-components/0805B104K500BD/15776052</t>
-  </si>
-  <si>
-    <t>TAJA105K016RNJ</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/products/detail/kyocera-avx/TAJA105K016RNJ/563757</t>
-  </si>
-  <si>
-    <t>TL8W9226M010C</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/products/detail/vishay-sprague/TL8W9226M010C/3883152</t>
-  </si>
-  <si>
-    <t>Zener_Diode</t>
-  </si>
-  <si>
-    <t>SD0805S040S0R5</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/products/detail/kyocera-avx/SD0805S040S0R5/3749489</t>
-  </si>
-  <si>
     <t>RC0805FR-075K1L</t>
   </si>
   <si>
@@ -224,13 +205,128 @@
   </si>
   <si>
     <t>https://www.digikey.com/en/products/detail/alpha-omega-semiconductor-inc/AO3400A/1855772</t>
+  </si>
+  <si>
+    <t>C1, C2</t>
+  </si>
+  <si>
+    <t>TLV75733PDBVR</t>
+  </si>
+  <si>
+    <t>1uF</t>
+  </si>
+  <si>
+    <t>TL3342F260QG</t>
+  </si>
+  <si>
+    <t>SW1, SW2</t>
+  </si>
+  <si>
+    <t>Enable, Boot</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/e-switch/TL3342F260QG/4029402</t>
+  </si>
+  <si>
+    <t>CRS08(TE85L,Q,M)</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/toshiba-semiconductor-and-storage/CRS08-TE85L-Q-M/871563?s=N4IgjCBcoGwJxVAYygMwIYBsDOBTANCAPZQDaIALAAxwDMdIAuoQA4AuUIAymwE4CWAOwDmIAL6EArAHYqiECkgYcBEADdBUPgFdVJSOWpVa0gBxNWHSNz5DREkHDAV5i5XkL7ykyVQoRCCh9JBECKOCpJECkAJlMwAPAwOGlfCxB2Th4BEXFCGKppCGgFNCwPYjIQWioAAgA1aOqYhqbaSVbAusbAjp6QX06QGG70zOsAVUF%2BNgB5VABZXHRsbV5cPJAYmJhi5DKVTyraEdqAW3ragAFasAA6DoBBMasQAGEibRZMXAATKZm8yWKzWGwcAFoYq4tLxdEcDAMmGJkUA</t>
+  </si>
+  <si>
+    <t>QBLP631-R5-2897</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/qt-brightek-qtb/QBLP631-R5-2897/23026393</t>
+  </si>
+  <si>
+    <t>USB_C_Receptacle_USB2.0_16P</t>
+  </si>
+  <si>
+    <t>USB4085-GF-A</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/gct/USB4085-GF-A/9859662?s=N4IgTCBcDaIOIGEAqACAqgZQEIBYAMAHAKwC0cAYiQIIgC6AvkA</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/w%C3%BCrth-elektronik/61300411121/4846827</t>
+  </si>
+  <si>
+    <t>691137710002</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/w%C3%BCrth-elektronik/691137710002/6644051</t>
+  </si>
+  <si>
+    <t>PJ-063AH</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/same-sky-formerly-cui-devices/PJ-063AH/2161208</t>
+  </si>
+  <si>
+    <t>ESP32-S3-WROOM-1-N8R2</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/espressif-systems/ESP32-S3-WROOM-1-N8R2/15200058?s=N4IgjCBcpgLATFUBjKAzAhgGwM4FMAaEAeygG0QB2eAZgA47KQBdIgBwBcoQBlDgJwCWAOwDmIAL5EAnADYArEhCpImXIRLkQ9eQAZZuluy6ReAkeKkhpdWEpVr8RUpArzYdedIisQnbnxCYpJEALSI0MpQAgCuGi5uLBJWERR4OGw08KE4NKEA6gBKAPLFALKhPhJAA</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/texas-instruments/TLV75733PDBVR/9343364</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/ceva-technologies-inc/BNO086/14114190</t>
+  </si>
+  <si>
+    <t>Total Price</t>
+  </si>
+  <si>
+    <t>Price Per Unit</t>
+  </si>
+  <si>
+    <t>Total Per Board</t>
+  </si>
+  <si>
+    <t>CL21B105KAFNNNE</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/samsung-electro-mechanics/CL21B105KAFNNNE/3886724</t>
+  </si>
+  <si>
+    <t>CL21B104KBCNNNC</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/samsung-electro-mechanics/CL21B104KBCNNNC/3886661</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/samsung-electro-mechanics/CL21A106KOQNNNE/3886754</t>
+  </si>
+  <si>
+    <t>CL21A106KOQNNNE</t>
+  </si>
+  <si>
+    <t>Maximum Price</t>
+  </si>
+  <si>
+    <t>Ratings:
+Resistors, Capacitors: 
+   • Vmax &gt;= 10V
+   • Imax &gt;= 1A
+   • Tolerance &lt;= +-10%</t>
+  </si>
+  <si>
+    <t>J4</t>
+  </si>
+  <si>
+    <t>Schottky_Diode</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="7" formatCode="&quot;$&quot;#,##0.00_);\(&quot;$&quot;#,##0.00\)"/>
+  </numFmts>
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -369,6 +465,33 @@
       <u/>
       <sz val="12"/>
       <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="20"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -890,7 +1013,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -910,12 +1033,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -925,17 +1042,42 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="20" xfId="42" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="21" xfId="42" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="7" fontId="19" fillId="0" borderId="20" xfId="42" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="7" fontId="19" fillId="0" borderId="21" xfId="42" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="7" fontId="0" fillId="0" borderId="20" xfId="42" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="7" fontId="0" fillId="0" borderId="21" xfId="42" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="7" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="43">
@@ -997,9 +1139,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1037,7 +1179,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1143,7 +1285,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1285,400 +1427,613 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FE4D61E-8A41-6646-9D5A-E2AE8EAB4DC9}">
-  <dimension ref="A1:F22"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FE4D61E-8A41-6646-9D5A-E2AE8EAB4DC9}">
+  <dimension ref="B2:I33"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.1640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.83203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="52.33203125" customWidth="1"/>
-    <col min="6" max="6" width="21.5" customWidth="1"/>
+    <col min="1" max="1" width="6.75" customWidth="1"/>
+    <col min="2" max="2" width="20.375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.75" customWidth="1"/>
+    <col min="4" max="4" width="28.5" customWidth="1"/>
+    <col min="5" max="5" width="23.125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="46.125" customWidth="1"/>
+    <col min="7" max="7" width="13.75" customWidth="1"/>
+    <col min="8" max="8" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="17" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+    <row r="2" spans="2:9" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="20" t="s">
+        <v>79</v>
+      </c>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+    </row>
+    <row r="3" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+    </row>
+    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B4" s="20"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="20"/>
+    </row>
+    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B5" s="20"/>
+      <c r="C5" s="20"/>
+      <c r="D5" s="20"/>
+      <c r="E5" s="20"/>
+    </row>
+    <row r="6" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B6" s="18"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="18"/>
+      <c r="E6" s="18"/>
+    </row>
+    <row r="7" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B7" s="18"/>
+      <c r="C7" s="18"/>
+      <c r="D7" s="18"/>
+      <c r="E7" s="18"/>
+    </row>
+    <row r="8" spans="2:9" ht="26.25" x14ac:dyDescent="0.4">
+      <c r="D8" s="21" t="s">
+        <v>78</v>
+      </c>
+      <c r="E8" s="21"/>
+      <c r="F8" s="21"/>
+    </row>
+    <row r="9" spans="2:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="10" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B10" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C10" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D10" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E10" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="11" spans="2:9" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B11" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11" s="6">
+        <v>6</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="F11" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="G11" s="15">
+        <v>0.1</v>
+      </c>
+      <c r="H11" s="13">
+        <f t="shared" ref="H11" si="0">G11*C11</f>
+        <v>0.60000000000000009</v>
+      </c>
+      <c r="I11" s="7"/>
+    </row>
+    <row r="12" spans="2:9" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B12" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="C12" s="6">
+        <v>2</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="F12" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="G12" s="15">
+        <v>0.1</v>
+      </c>
+      <c r="H12" s="13">
+        <f>G12*C12</f>
+        <v>0.2</v>
+      </c>
+      <c r="I12" s="7"/>
+    </row>
+    <row r="13" spans="2:9" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B13" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C13" s="6">
+        <v>2</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="F13" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="G13" s="15">
+        <v>0.1</v>
+      </c>
+      <c r="H13" s="13">
+        <f t="shared" ref="H13" si="1">G13*C13</f>
+        <v>0.2</v>
+      </c>
+      <c r="I13" s="7"/>
+    </row>
+    <row r="14" spans="2:9" ht="173.25" x14ac:dyDescent="0.25">
+      <c r="B14" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C14" s="6">
+        <v>2</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="F14" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="G14" s="15">
+        <v>0.7</v>
+      </c>
+      <c r="H14" s="13">
+        <f>G14*C14</f>
+        <v>1.4</v>
+      </c>
+      <c r="I14" s="7"/>
+    </row>
+    <row r="15" spans="2:9" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B15" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C15" s="6">
+        <v>1</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F15" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="G15" s="15">
+        <v>0.23</v>
+      </c>
+      <c r="H15" s="13">
+        <f>G15*C15</f>
+        <v>0.23</v>
+      </c>
+      <c r="I15" s="7"/>
+    </row>
+    <row r="16" spans="2:9" ht="63" x14ac:dyDescent="0.25">
+      <c r="B16" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="C16" s="6">
+        <v>1</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="F16" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="G16" s="15">
+        <v>0.91</v>
+      </c>
+      <c r="H16" s="13">
+        <f t="shared" ref="H16:H28" si="2">G16*C16</f>
+        <v>0.91</v>
+      </c>
+      <c r="I16" s="7"/>
+    </row>
+    <row r="17" spans="2:9" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B17" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C17" s="6">
+        <v>1</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E17" s="6">
+        <v>61300411121</v>
+      </c>
+      <c r="F17" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="G17" s="15">
+        <v>0.19</v>
+      </c>
+      <c r="H17" s="13">
+        <f t="shared" si="2"/>
+        <v>0.19</v>
+      </c>
+      <c r="I17" s="7"/>
+    </row>
+    <row r="18" spans="2:9" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B18" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C18" s="6">
+        <v>1</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="F18" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="G18" s="15">
+        <v>1.49</v>
+      </c>
+      <c r="H18" s="13">
+        <f t="shared" si="2"/>
+        <v>1.49</v>
+      </c>
+      <c r="I18" s="7"/>
+    </row>
+    <row r="19" spans="2:9" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B19" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C19" s="6">
+        <v>1</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E19" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="F19" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="G19" s="15">
+        <v>0.41</v>
+      </c>
+      <c r="H19" s="13">
+        <f t="shared" si="2"/>
+        <v>0.41</v>
+      </c>
+      <c r="I19" s="7"/>
+    </row>
+    <row r="20" spans="2:9" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B20" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C20" s="6">
+        <v>1</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F20" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="G20" s="15">
+        <v>0.52</v>
+      </c>
+      <c r="H20" s="13">
+        <f t="shared" si="2"/>
+        <v>0.52</v>
+      </c>
+      <c r="I20" s="7"/>
+    </row>
+    <row r="21" spans="2:9" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="B21" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C21" s="6">
+        <v>1</v>
+      </c>
+      <c r="D21" s="6">
+        <v>220</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="F21" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="G21" s="15">
+        <v>0.1</v>
+      </c>
+      <c r="H21" s="13">
+        <f>G21*C21</f>
+        <v>0.1</v>
+      </c>
+      <c r="I21" s="7"/>
+    </row>
+    <row r="22" spans="2:9" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B22" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C22" s="6">
+        <v>1</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="F22" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="G22" s="15">
+        <v>0.1</v>
+      </c>
+      <c r="H22" s="13">
+        <f>G22*C22</f>
+        <v>0.1</v>
+      </c>
+      <c r="I22" s="7"/>
+    </row>
+    <row r="23" spans="2:9" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B23" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C23" s="6">
+        <v>4</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E23" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F23" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="G23" s="15">
+        <v>0.1</v>
+      </c>
+      <c r="H23" s="13">
+        <f>G23*C23</f>
+        <v>0.4</v>
+      </c>
+      <c r="I23" s="7"/>
+    </row>
+    <row r="24" spans="2:9" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B24" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C24" s="6">
+        <v>2</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E24" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="F24" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="G24" s="15">
+        <v>0.1</v>
+      </c>
+      <c r="H24" s="13">
+        <f>G24*C24</f>
+        <v>0.2</v>
+      </c>
+      <c r="I24" s="7"/>
+    </row>
+    <row r="25" spans="2:9" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B25" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C25" s="6">
+        <v>5</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="F25" s="11" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" ht="34" x14ac:dyDescent="0.2">
-      <c r="A2" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="B2" s="6">
+      <c r="G25" s="15">
+        <v>0.1</v>
+      </c>
+      <c r="H25" s="13">
+        <f>G25*C25</f>
+        <v>0.5</v>
+      </c>
+      <c r="I25" s="7"/>
+    </row>
+    <row r="26" spans="2:9" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B26" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C26" s="6">
+        <v>2</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="E26" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="F26" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="G26" s="15">
+        <v>0.59</v>
+      </c>
+      <c r="H26" s="13">
+        <f t="shared" si="2"/>
+        <v>1.18</v>
+      </c>
+      <c r="I26" s="7"/>
+    </row>
+    <row r="27" spans="2:9" ht="126" x14ac:dyDescent="0.25">
+      <c r="B27" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C27" s="6">
         <v>1</v>
       </c>
-      <c r="C2" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="E2" s="15" t="s">
-        <v>51</v>
-      </c>
-      <c r="F2" s="9" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="34" x14ac:dyDescent="0.2">
-      <c r="A3" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="6">
+      <c r="D27" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="F27" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="G27" s="15">
+        <v>5.88</v>
+      </c>
+      <c r="H27" s="13">
+        <f t="shared" si="2"/>
+        <v>5.88</v>
+      </c>
+      <c r="I27" s="7"/>
+    </row>
+    <row r="28" spans="2:9" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B28" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C28" s="6">
         <v>1</v>
       </c>
-      <c r="C3" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="D3" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="E3" s="15" t="s">
-        <v>53</v>
-      </c>
-      <c r="F3" s="9" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="34" x14ac:dyDescent="0.2">
-      <c r="A4" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" s="6">
-        <v>6</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="E4" s="15" t="s">
-        <v>49</v>
-      </c>
-      <c r="F4" s="9"/>
-    </row>
-    <row r="5" spans="1:6" ht="34" x14ac:dyDescent="0.2">
-      <c r="A5" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="B5" s="6">
-        <v>2</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="E5" s="15" t="s">
+      <c r="D28" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="F5" s="9"/>
-    </row>
-    <row r="6" spans="1:6" ht="34" x14ac:dyDescent="0.2">
-      <c r="A6" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" s="6">
-        <v>2</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="E6" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="F6" s="9"/>
-    </row>
-    <row r="7" spans="1:6" ht="17" x14ac:dyDescent="0.2">
-      <c r="A7" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" s="6">
+      <c r="E28" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="F28" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="G28" s="15">
+        <v>0.34</v>
+      </c>
+      <c r="H28" s="13">
+        <f t="shared" si="2"/>
+        <v>0.34</v>
+      </c>
+      <c r="I28" s="7"/>
+    </row>
+    <row r="29" spans="2:9" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B29" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C29" s="9">
         <v>1</v>
       </c>
-      <c r="C7" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D7" s="7"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="9"/>
-    </row>
-    <row r="8" spans="1:6" ht="17" x14ac:dyDescent="0.2">
-      <c r="A8" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8" s="6">
-        <v>1</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D8" s="7"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="9"/>
-    </row>
-    <row r="9" spans="1:6" ht="17" x14ac:dyDescent="0.2">
-      <c r="A9" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B9" s="6">
-        <v>1</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="D9" s="7"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="9"/>
-    </row>
-    <row r="10" spans="1:6" ht="17" x14ac:dyDescent="0.2">
-      <c r="A10" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="B10" s="6">
-        <v>1</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="D10" s="7"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="9"/>
-    </row>
-    <row r="11" spans="1:6" ht="17" x14ac:dyDescent="0.2">
-      <c r="A11" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="B11" s="6">
-        <v>1</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="D11" s="7"/>
-      <c r="E11" s="8"/>
-      <c r="F11" s="9"/>
-    </row>
-    <row r="12" spans="1:6" ht="34" x14ac:dyDescent="0.2">
-      <c r="A12" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B12" s="6">
-        <v>1</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="E12" s="15" t="s">
-        <v>67</v>
-      </c>
-      <c r="F12" s="9"/>
-    </row>
-    <row r="13" spans="1:6" ht="34" x14ac:dyDescent="0.2">
-      <c r="A13" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="B13" s="6">
-        <v>2</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="D13" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="E13" s="15" t="s">
-        <v>58</v>
-      </c>
-      <c r="F13" s="9"/>
-    </row>
-    <row r="14" spans="1:6" ht="34" x14ac:dyDescent="0.2">
-      <c r="A14" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="B14" s="6">
-        <v>5</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="D14" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="E14" s="15" t="s">
-        <v>66</v>
-      </c>
-      <c r="F14" s="9"/>
-    </row>
-    <row r="15" spans="1:6" ht="34" x14ac:dyDescent="0.2">
-      <c r="A15" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B15" s="6">
-        <v>1</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="D15" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="E15" s="15" t="s">
-        <v>62</v>
-      </c>
-      <c r="F15" s="9"/>
-    </row>
-    <row r="16" spans="1:6" ht="34" x14ac:dyDescent="0.2">
-      <c r="A16" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="B16" s="6">
-        <v>4</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="D16" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="E16" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="F16" s="9"/>
-    </row>
-    <row r="17" spans="1:6" ht="34" x14ac:dyDescent="0.2">
-      <c r="A17" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="B17" s="6">
-        <v>1</v>
-      </c>
-      <c r="C17" s="6">
-        <v>220</v>
-      </c>
-      <c r="D17" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="E17" s="15" t="s">
-        <v>60</v>
-      </c>
-      <c r="F17" s="9"/>
-    </row>
-    <row r="18" spans="1:6" ht="17" x14ac:dyDescent="0.2">
-      <c r="A18" s="5" t="s">
+      <c r="D29" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="B18" s="6">
-        <v>1</v>
-      </c>
-      <c r="C18" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="D18" s="7"/>
-      <c r="E18" s="8"/>
-      <c r="F18" s="9"/>
-    </row>
-    <row r="19" spans="1:6" ht="17" x14ac:dyDescent="0.2">
-      <c r="A19" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="B19" s="6">
-        <v>1</v>
-      </c>
-      <c r="C19" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="D19" s="7"/>
-      <c r="E19" s="8"/>
-      <c r="F19" s="9"/>
-    </row>
-    <row r="20" spans="1:6" ht="17" x14ac:dyDescent="0.2">
-      <c r="A20" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="B20" s="6">
-        <v>1</v>
-      </c>
-      <c r="C20" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="D20" s="7"/>
-      <c r="E20" s="8"/>
-      <c r="F20" s="9"/>
-    </row>
-    <row r="21" spans="1:6" ht="17" x14ac:dyDescent="0.2">
-      <c r="A21" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="B21" s="6">
-        <v>1</v>
-      </c>
-      <c r="C21" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="D21" s="7"/>
-      <c r="E21" s="8"/>
-      <c r="F21" s="9"/>
-    </row>
-    <row r="22" spans="1:6" ht="18" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="B22" s="11">
-        <v>1</v>
-      </c>
-      <c r="C22" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="D22" s="12"/>
-      <c r="E22" s="13"/>
-      <c r="F22" s="14"/>
+      <c r="E29" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="F29" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="G29" s="16">
+        <v>13.93</v>
+      </c>
+      <c r="H29" s="14">
+        <f>G29*C29</f>
+        <v>13.93</v>
+      </c>
+      <c r="I29" s="10"/>
+    </row>
+    <row r="33" spans="6:8" ht="26.25" x14ac:dyDescent="0.4">
+      <c r="F33" s="22" t="s">
+        <v>71</v>
+      </c>
+      <c r="G33" s="22"/>
+      <c r="H33" s="19">
+        <f>SUM(H11:H29)</f>
+        <v>28.78</v>
+      </c>
     </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B2:E5"/>
+    <mergeCell ref="D8:F8"/>
+    <mergeCell ref="F33:G33"/>
+  </mergeCells>
   <hyperlinks>
-    <hyperlink ref="E4" r:id="rId1" xr:uid="{22501009-131F-F34F-BD7F-EF905D9EECAF}"/>
-    <hyperlink ref="E2" r:id="rId2" xr:uid="{E71D0461-49E1-2149-B7CF-2F41909EACE2}"/>
-    <hyperlink ref="E3" r:id="rId3" xr:uid="{6979F835-A472-B04D-8947-920B68983C00}"/>
-    <hyperlink ref="E6" r:id="rId4" xr:uid="{337159D0-61B0-334C-A8B6-0319F7D57071}"/>
-    <hyperlink ref="E5" r:id="rId5" xr:uid="{3A98A724-3E45-AE47-923C-262A9EC1BCB5}"/>
-    <hyperlink ref="E13" r:id="rId6" xr:uid="{3ED07C84-AED5-5046-8009-9E8FC6343093}"/>
-    <hyperlink ref="E17" r:id="rId7" xr:uid="{B4DDEDFF-83AD-DE44-A720-01E9A6218C06}"/>
-    <hyperlink ref="E15" r:id="rId8" xr:uid="{64BFA3C5-0E31-3E44-AEFE-8E777214AE83}"/>
-    <hyperlink ref="E16" r:id="rId9" xr:uid="{ECAAFF86-F2E3-3B4E-BD0A-D874868F98EE}"/>
-    <hyperlink ref="E14" r:id="rId10" xr:uid="{46EF1F3A-9D57-D144-B01C-B8CB11D0619B}"/>
-    <hyperlink ref="E12" r:id="rId11" xr:uid="{91FC7FC0-C192-2F4A-82CF-0FD28D70D440}"/>
+    <hyperlink ref="F20" r:id="rId1" xr:uid="{91FC7FC0-C192-2F4A-82CF-0FD28D70D440}"/>
+    <hyperlink ref="F26" r:id="rId2" xr:uid="{3C9AB0B8-62AF-4F87-B3D1-873CD675C787}"/>
+    <hyperlink ref="F14" r:id="rId3" display="https://www.digikey.com/en/products/detail/toshiba-semiconductor-and-storage/CRS08-TE85L-Q-M/871563?s=N4IgjCBcoGwJxVAYygMwIYBsDOBTANCAPZQDaIALAAxwDMdIAuoQA4AuUIAymwE4CWAOwDmIAL6EArAHYqiECkgYcBEADdBUPgFdVJSOWpVa0gBxNWHSNz5DREkHDAV5i5XkL7ykyVQoRCCh9JBECKOCpJECkAJlMwAPAwOGlfCxB2Th4BEXFCGKppCGgFNCwPYjIQWioAAgA1aOqYhqbaSVbAusbAjp6QX06QGG70zOsAVUF%2BNgB5VABZXHRsbV5cPJAYmJhi5DKVTyraEdqAW3ragAFasAA6DoBBMasQAGEibRZMXAATKZm8yWKzWGwcAFoYq4tLxdEcDAMmGJkUA" xr:uid="{8F52F645-C15D-475D-A267-4C6E7D315F38}"/>
+    <hyperlink ref="F15" r:id="rId4" xr:uid="{311B3AB0-3265-41D5-9DC9-F4701ABE5C46}"/>
+    <hyperlink ref="F16" r:id="rId5" xr:uid="{0CADED76-C55B-491D-B56D-7B9C2E215846}"/>
+    <hyperlink ref="F17" r:id="rId6" xr:uid="{1C87D9BC-E94A-4598-B0E9-B3B8EB790AE8}"/>
+    <hyperlink ref="F19" r:id="rId7" xr:uid="{50829CBF-7D09-4245-A34F-BEC84C379753}"/>
+    <hyperlink ref="F18" r:id="rId8" xr:uid="{11C72523-FD00-4FB3-BE9D-E75886251EA5}"/>
+    <hyperlink ref="F27" r:id="rId9" display="https://www.digikey.com/en/products/detail/espressif-systems/ESP32-S3-WROOM-1-N8R2/15200058?s=N4IgjCBcpgLATFUBjKAzAhgGwM4FMAaEAeygG0QB2eAZgA47KQBdIgBwBcoQBlDgJwCWAOwDmIAL5EAnADYArEhCpImXIRLkQ9eQAZZuluy6ReAkeKkhpdWEpVr8RUpArzYdedIisQnbnxCYpJEALSI0MpQAgCuGi5uLBJWERR4OGw08KE4NKEA6gBKAPLFALKhPhJAA" xr:uid="{EE4D866C-5F9C-4298-A67E-DDE6B25EE229}"/>
+    <hyperlink ref="F28" r:id="rId10" xr:uid="{41BFA31B-E2BB-47BF-A00F-F73F3C52D952}"/>
+    <hyperlink ref="F29" r:id="rId11" xr:uid="{B57C1A14-D5E2-493D-B573-5A2C10E0FA37}"/>
+    <hyperlink ref="F13" r:id="rId12" xr:uid="{DAF0E7CF-0B00-472D-AD7F-083EDC4A3C11}"/>
+    <hyperlink ref="F12" r:id="rId13" xr:uid="{5037AFDF-5497-4CCA-9114-4D0481773CBA}"/>
+    <hyperlink ref="F11" r:id="rId14" xr:uid="{F66DC830-E623-4FF0-B1A4-A9DDF6642F7D}"/>
+    <hyperlink ref="F24" r:id="rId15" xr:uid="{DB02A26D-A2F0-4DBD-ACF0-BF87BEB7D264}"/>
+    <hyperlink ref="F21" r:id="rId16" xr:uid="{3B3F9571-6F5C-47AA-90ED-896C511E55F3}"/>
+    <hyperlink ref="F22" r:id="rId17" xr:uid="{E95100A1-7BF1-40F0-BDEC-1F16D937F2C7}"/>
+    <hyperlink ref="F23" r:id="rId18" xr:uid="{42C9434C-B343-4B2A-80F3-106ED6DA912B}"/>
+    <hyperlink ref="F25" r:id="rId19" xr:uid="{8DCCBA24-FD10-45CE-87F0-8AAA09E69458}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId20"/>
+  <legacyDrawing r:id="rId21"/>
 </worksheet>
 </file>
</xml_diff>